<commit_message>
2025.01.04_2 deleted obsolete tidyverse part from the end
</commit_message>
<xml_diff>
--- a/data_codebook.xlsx
+++ b/data_codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gustavosplmoura/Library/Mobile Documents/com~apple~CloudDocs/Medicina/Biblioteca/Research/Data Science/Data Science/PROJECTS/DVEP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664BD572-A1A2-DF46-BA88-D9D4889D2C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{809C7A70-B402-C84A-B6D7-DBC4C011C2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20140" xr2:uid="{64E364A7-669F-4B4E-A75E-FD8B217DB5CF}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10123" uniqueCount="5732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10125" uniqueCount="5733">
   <si>
     <t>variable</t>
   </si>
@@ -17514,10 +17514,13 @@
     <t>k</t>
   </si>
   <si>
-    <t>eleg_arm_1, 0 | 1visit_arm_1, 1 |2visit_arm_1, 2 | 3visit_arm_1, 3</t>
-  </si>
-  <si>
     <t>o</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>eleg_arm_1, 0 | 1visit_arm_1, 1 | 2visit_arm_1, 2 | 3visit_arm_1, 3</t>
   </si>
 </sst>
 </file>
@@ -18230,6 +18233,9 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C9BD1FE7-06E6-AF49-9672-E4E31AED68CC}" name="Table2" displayName="Table2" ref="A1:AA781" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A1:AA781" xr:uid="{C9BD1FE7-06E6-AF49-9672-E4E31AED68CC}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AA781">
+    <sortCondition ref="A1:A781"/>
+  </sortState>
   <tableColumns count="27">
     <tableColumn id="1" xr3:uid="{204E05AD-B324-584D-9052-1D5D7A5AF23C}" name="index" dataDxfId="30"/>
     <tableColumn id="2" xr3:uid="{E78D0B38-AC8A-0541-A7D9-8D9DE8100BFC}" name="variable" dataDxfId="29"/>
@@ -18593,7 +18599,7 @@
     <col min="10" max="10" width="13.19921875" customWidth="1"/>
     <col min="11" max="11" width="6.796875" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="99.796875" customWidth="1"/>
+    <col min="13" max="13" width="28.59765625" customWidth="1"/>
     <col min="15" max="15" width="34.3984375" customWidth="1"/>
     <col min="17" max="17" width="53.59765625" customWidth="1"/>
     <col min="18" max="18" width="8.19921875" customWidth="1"/>
@@ -18781,7 +18787,7 @@
         <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>5730</v>
+        <v>5732</v>
       </c>
       <c r="N3" t="s">
         <v>38</v>
@@ -19067,7 +19073,7 @@
         <v>72</v>
       </c>
       <c r="L8" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M8" t="s">
         <v>73</v>
@@ -19132,7 +19138,7 @@
         <v>72</v>
       </c>
       <c r="L9" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M9" t="s">
         <v>80</v>
@@ -19197,7 +19203,7 @@
         <v>72</v>
       </c>
       <c r="L10" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M10" t="s">
         <v>90</v>
@@ -19259,7 +19265,7 @@
         <v>72</v>
       </c>
       <c r="L11" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M11" t="s">
         <v>99</v>
@@ -19321,7 +19327,7 @@
         <v>72</v>
       </c>
       <c r="L12" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M12" t="s">
         <v>108</v>
@@ -19383,7 +19389,7 @@
         <v>72</v>
       </c>
       <c r="L13" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M13" t="s">
         <v>116</v>
@@ -19445,7 +19451,7 @@
         <v>72</v>
       </c>
       <c r="L14" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M14" t="s">
         <v>125</v>
@@ -19560,7 +19566,7 @@
         <v>72</v>
       </c>
       <c r="L16" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M16" t="s">
         <v>140</v>
@@ -19625,7 +19631,7 @@
         <v>72</v>
       </c>
       <c r="L17" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M17" t="s">
         <v>125</v>
@@ -19873,7 +19879,7 @@
         <v>72</v>
       </c>
       <c r="L21" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M21" t="s">
         <v>125</v>
@@ -19991,7 +19997,7 @@
         <v>72</v>
       </c>
       <c r="L23" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M23" t="s">
         <v>125</v>
@@ -20109,7 +20115,7 @@
         <v>72</v>
       </c>
       <c r="L25" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M25" t="s">
         <v>125</v>
@@ -20171,7 +20177,7 @@
         <v>72</v>
       </c>
       <c r="L26" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M26" t="s">
         <v>125</v>
@@ -20233,7 +20239,7 @@
         <v>72</v>
       </c>
       <c r="L27" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M27" t="s">
         <v>125</v>
@@ -20295,7 +20301,7 @@
         <v>72</v>
       </c>
       <c r="L28" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M28" t="s">
         <v>125</v>
@@ -20357,7 +20363,7 @@
         <v>72</v>
       </c>
       <c r="L29" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M29" t="s">
         <v>125</v>
@@ -20419,7 +20425,7 @@
         <v>72</v>
       </c>
       <c r="L30" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M30" t="s">
         <v>125</v>
@@ -20481,7 +20487,7 @@
         <v>72</v>
       </c>
       <c r="L31" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M31" t="s">
         <v>125</v>
@@ -20543,7 +20549,7 @@
         <v>72</v>
       </c>
       <c r="L32" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M32" t="s">
         <v>125</v>
@@ -20605,7 +20611,7 @@
         <v>72</v>
       </c>
       <c r="L33" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M33" t="s">
         <v>125</v>
@@ -20667,7 +20673,7 @@
         <v>72</v>
       </c>
       <c r="L34" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M34" t="s">
         <v>125</v>
@@ -20729,7 +20735,7 @@
         <v>72</v>
       </c>
       <c r="L35" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M35" t="s">
         <v>125</v>
@@ -20791,7 +20797,7 @@
         <v>72</v>
       </c>
       <c r="L36" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M36" t="s">
         <v>125</v>
@@ -20853,7 +20859,7 @@
         <v>72</v>
       </c>
       <c r="L37" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M37" t="s">
         <v>125</v>
@@ -20918,7 +20924,7 @@
         <v>72</v>
       </c>
       <c r="L38" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M38" t="s">
         <v>125</v>
@@ -20980,7 +20986,7 @@
         <v>72</v>
       </c>
       <c r="L39" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M39" t="s">
         <v>125</v>
@@ -21042,7 +21048,7 @@
         <v>72</v>
       </c>
       <c r="L40" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M40" t="s">
         <v>125</v>
@@ -21104,7 +21110,7 @@
         <v>72</v>
       </c>
       <c r="L41" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M41" t="s">
         <v>125</v>
@@ -21166,7 +21172,7 @@
         <v>72</v>
       </c>
       <c r="L42" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M42" t="s">
         <v>125</v>
@@ -21228,7 +21234,7 @@
         <v>72</v>
       </c>
       <c r="L43" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M43" t="s">
         <v>125</v>
@@ -21290,7 +21296,7 @@
         <v>72</v>
       </c>
       <c r="L44" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M44" t="s">
         <v>125</v>
@@ -21352,7 +21358,7 @@
         <v>72</v>
       </c>
       <c r="L45" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M45" t="s">
         <v>125</v>
@@ -21414,7 +21420,7 @@
         <v>72</v>
       </c>
       <c r="L46" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M46" t="s">
         <v>125</v>
@@ -21476,7 +21482,7 @@
         <v>72</v>
       </c>
       <c r="L47" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M47" t="s">
         <v>125</v>
@@ -21538,7 +21544,7 @@
         <v>72</v>
       </c>
       <c r="L48" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M48" t="s">
         <v>125</v>
@@ -21600,7 +21606,7 @@
         <v>72</v>
       </c>
       <c r="L49" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M49" t="s">
         <v>125</v>
@@ -21662,7 +21668,7 @@
         <v>72</v>
       </c>
       <c r="L50" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M50" t="s">
         <v>125</v>
@@ -21724,7 +21730,7 @@
         <v>72</v>
       </c>
       <c r="L51" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M51" t="s">
         <v>125</v>
@@ -22013,7 +22019,7 @@
         <v>72</v>
       </c>
       <c r="L56" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M56" t="s">
         <v>423</v>
@@ -22075,7 +22081,7 @@
         <v>432</v>
       </c>
       <c r="L57" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M57" t="s">
         <v>125</v>
@@ -22137,7 +22143,7 @@
         <v>432</v>
       </c>
       <c r="L58" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M58" t="s">
         <v>125</v>
@@ -22199,7 +22205,7 @@
         <v>432</v>
       </c>
       <c r="L59" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M59" t="s">
         <v>125</v>
@@ -22261,7 +22267,7 @@
         <v>72</v>
       </c>
       <c r="L60" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M60" t="s">
         <v>125</v>
@@ -22323,7 +22329,7 @@
         <v>72</v>
       </c>
       <c r="L61" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M61" t="s">
         <v>465</v>
@@ -22444,7 +22450,7 @@
         <v>72</v>
       </c>
       <c r="L63" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M63" t="s">
         <v>125</v>
@@ -22509,7 +22515,7 @@
         <v>72</v>
       </c>
       <c r="L64" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M64" t="s">
         <v>125</v>
@@ -22633,7 +22639,7 @@
         <v>72</v>
       </c>
       <c r="L66" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M66" t="s">
         <v>125</v>
@@ -22695,7 +22701,7 @@
         <v>72</v>
       </c>
       <c r="L67" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M67" t="s">
         <v>125</v>
@@ -22757,7 +22763,7 @@
         <v>72</v>
       </c>
       <c r="L68" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M68" t="s">
         <v>125</v>
@@ -22872,7 +22878,7 @@
         <v>72</v>
       </c>
       <c r="L70" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M70" t="s">
         <v>125</v>
@@ -22934,7 +22940,7 @@
         <v>72</v>
       </c>
       <c r="L71" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M71" t="s">
         <v>125</v>
@@ -23052,7 +23058,7 @@
         <v>72</v>
       </c>
       <c r="L73" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M73" t="s">
         <v>125</v>
@@ -23114,7 +23120,7 @@
         <v>72</v>
       </c>
       <c r="L74" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M74" t="s">
         <v>557</v>
@@ -23176,7 +23182,7 @@
         <v>28</v>
       </c>
       <c r="L75" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="P75" t="s">
         <v>566</v>
@@ -23291,7 +23297,7 @@
         <v>72</v>
       </c>
       <c r="L77" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M77" t="s">
         <v>578</v>
@@ -23353,7 +23359,7 @@
         <v>72</v>
       </c>
       <c r="L78" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M78" t="s">
         <v>125</v>
@@ -23545,7 +23551,7 @@
         <v>72</v>
       </c>
       <c r="L81" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M81" t="s">
         <v>578</v>
@@ -23964,7 +23970,7 @@
         <v>72</v>
       </c>
       <c r="L88" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M88" t="s">
         <v>664</v>
@@ -24082,7 +24088,7 @@
         <v>72</v>
       </c>
       <c r="L90" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M90" t="s">
         <v>578</v>
@@ -24144,7 +24150,7 @@
         <v>28</v>
       </c>
       <c r="L91" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q91" t="s">
         <v>567</v>
@@ -24200,7 +24206,7 @@
         <v>72</v>
       </c>
       <c r="L92" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M92" t="s">
         <v>693</v>
@@ -24265,7 +24271,7 @@
         <v>72</v>
       </c>
       <c r="L93" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M93" t="s">
         <v>702</v>
@@ -24330,7 +24336,7 @@
         <v>72</v>
       </c>
       <c r="L94" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M94" t="s">
         <v>711</v>
@@ -24395,7 +24401,7 @@
         <v>72</v>
       </c>
       <c r="L95" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M95" t="s">
         <v>711</v>
@@ -24460,7 +24466,7 @@
         <v>72</v>
       </c>
       <c r="L96" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M96" t="s">
         <v>711</v>
@@ -24525,7 +24531,7 @@
         <v>72</v>
       </c>
       <c r="L97" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M97" t="s">
         <v>711</v>
@@ -24590,7 +24596,7 @@
         <v>72</v>
       </c>
       <c r="L98" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M98" t="s">
         <v>711</v>
@@ -24655,7 +24661,7 @@
         <v>72</v>
       </c>
       <c r="L99" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M99" t="s">
         <v>711</v>
@@ -24720,7 +24726,7 @@
         <v>72</v>
       </c>
       <c r="L100" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M100" t="s">
         <v>711</v>
@@ -24785,7 +24791,7 @@
         <v>72</v>
       </c>
       <c r="L101" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M101" t="s">
         <v>768</v>
@@ -24850,7 +24856,7 @@
         <v>72</v>
       </c>
       <c r="L102" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M102" t="s">
         <v>768</v>
@@ -24915,7 +24921,7 @@
         <v>72</v>
       </c>
       <c r="L103" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M103" t="s">
         <v>768</v>
@@ -24980,7 +24986,7 @@
         <v>72</v>
       </c>
       <c r="L104" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M104" t="s">
         <v>768</v>
@@ -25045,7 +25051,7 @@
         <v>72</v>
       </c>
       <c r="L105" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M105" t="s">
         <v>768</v>
@@ -25110,7 +25116,7 @@
         <v>72</v>
       </c>
       <c r="L106" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M106" t="s">
         <v>693</v>
@@ -25175,7 +25181,7 @@
         <v>72</v>
       </c>
       <c r="L107" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M107" t="s">
         <v>693</v>
@@ -25240,7 +25246,7 @@
         <v>72</v>
       </c>
       <c r="L108" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M108" t="s">
         <v>693</v>
@@ -25305,7 +25311,7 @@
         <v>72</v>
       </c>
       <c r="L109" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M109" t="s">
         <v>693</v>
@@ -25370,7 +25376,7 @@
         <v>72</v>
       </c>
       <c r="L110" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M110" t="s">
         <v>693</v>
@@ -25435,7 +25441,7 @@
         <v>72</v>
       </c>
       <c r="L111" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M111" t="s">
         <v>693</v>
@@ -25500,7 +25506,7 @@
         <v>72</v>
       </c>
       <c r="L112" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M112" t="s">
         <v>693</v>
@@ -25565,7 +25571,7 @@
         <v>72</v>
       </c>
       <c r="L113" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M113" t="s">
         <v>693</v>
@@ -25630,7 +25636,7 @@
         <v>72</v>
       </c>
       <c r="L114" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M114" t="s">
         <v>693</v>
@@ -25695,7 +25701,7 @@
         <v>72</v>
       </c>
       <c r="L115" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M115" t="s">
         <v>693</v>
@@ -25760,7 +25766,7 @@
         <v>72</v>
       </c>
       <c r="L116" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M116" t="s">
         <v>693</v>
@@ -25825,7 +25831,7 @@
         <v>72</v>
       </c>
       <c r="L117" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M117" t="s">
         <v>896</v>
@@ -25890,7 +25896,7 @@
         <v>72</v>
       </c>
       <c r="L118" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M118" t="s">
         <v>905</v>
@@ -26400,7 +26406,7 @@
         <v>72</v>
       </c>
       <c r="L127" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M127" t="s">
         <v>578</v>
@@ -26462,7 +26468,7 @@
         <v>28</v>
       </c>
       <c r="L128" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q128" t="s">
         <v>567</v>
@@ -26518,7 +26524,7 @@
         <v>72</v>
       </c>
       <c r="L129" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M129" t="s">
         <v>981</v>
@@ -26583,7 +26589,7 @@
         <v>72</v>
       </c>
       <c r="L130" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M130" t="s">
         <v>981</v>
@@ -26648,7 +26654,7 @@
         <v>72</v>
       </c>
       <c r="L131" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M131" t="s">
         <v>981</v>
@@ -26713,7 +26719,7 @@
         <v>72</v>
       </c>
       <c r="L132" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M132" t="s">
         <v>981</v>
@@ -26778,7 +26784,7 @@
         <v>72</v>
       </c>
       <c r="L133" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M133" t="s">
         <v>981</v>
@@ -26843,7 +26849,7 @@
         <v>72</v>
       </c>
       <c r="L134" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M134" t="s">
         <v>981</v>
@@ -26908,7 +26914,7 @@
         <v>72</v>
       </c>
       <c r="L135" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M135" t="s">
         <v>981</v>
@@ -26973,7 +26979,7 @@
         <v>72</v>
       </c>
       <c r="L136" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M136" t="s">
         <v>981</v>
@@ -27038,7 +27044,7 @@
         <v>72</v>
       </c>
       <c r="L137" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M137" t="s">
         <v>981</v>
@@ -27103,7 +27109,7 @@
         <v>72</v>
       </c>
       <c r="L138" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M138" t="s">
         <v>981</v>
@@ -27168,7 +27174,7 @@
         <v>72</v>
       </c>
       <c r="L139" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M139" t="s">
         <v>981</v>
@@ -27233,7 +27239,7 @@
         <v>72</v>
       </c>
       <c r="L140" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M140" t="s">
         <v>981</v>
@@ -27298,7 +27304,7 @@
         <v>72</v>
       </c>
       <c r="L141" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M141" t="s">
         <v>981</v>
@@ -27363,7 +27369,7 @@
         <v>72</v>
       </c>
       <c r="L142" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M142" t="s">
         <v>981</v>
@@ -27428,7 +27434,7 @@
         <v>72</v>
       </c>
       <c r="L143" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M143" t="s">
         <v>981</v>
@@ -27493,7 +27499,7 @@
         <v>72</v>
       </c>
       <c r="L144" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M144" t="s">
         <v>981</v>
@@ -27558,7 +27564,7 @@
         <v>72</v>
       </c>
       <c r="L145" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M145" t="s">
         <v>981</v>
@@ -27623,7 +27629,7 @@
         <v>72</v>
       </c>
       <c r="L146" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M146" t="s">
         <v>981</v>
@@ -27688,7 +27694,7 @@
         <v>72</v>
       </c>
       <c r="L147" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M147" t="s">
         <v>981</v>
@@ -27753,7 +27759,7 @@
         <v>72</v>
       </c>
       <c r="L148" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M148" t="s">
         <v>981</v>
@@ -27818,7 +27824,7 @@
         <v>72</v>
       </c>
       <c r="L149" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M149" t="s">
         <v>981</v>
@@ -28107,7 +28113,7 @@
         <v>72</v>
       </c>
       <c r="L154" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M154" t="s">
         <v>578</v>
@@ -28169,7 +28175,7 @@
         <v>28</v>
       </c>
       <c r="L155" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q155" t="s">
         <v>567</v>
@@ -28225,7 +28231,7 @@
         <v>72</v>
       </c>
       <c r="L156" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M156" t="s">
         <v>1188</v>
@@ -28290,7 +28296,7 @@
         <v>72</v>
       </c>
       <c r="L157" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M157" t="s">
         <v>1195</v>
@@ -28355,7 +28361,7 @@
         <v>72</v>
       </c>
       <c r="L158" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M158" t="s">
         <v>1202</v>
@@ -28420,7 +28426,7 @@
         <v>72</v>
       </c>
       <c r="L159" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M159" t="s">
         <v>1209</v>
@@ -28485,7 +28491,7 @@
         <v>72</v>
       </c>
       <c r="L160" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M160" t="s">
         <v>1216</v>
@@ -28550,7 +28556,7 @@
         <v>72</v>
       </c>
       <c r="L161" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M161" t="s">
         <v>1223</v>
@@ -28615,7 +28621,7 @@
         <v>72</v>
       </c>
       <c r="L162" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M162" t="s">
         <v>1230</v>
@@ -28680,7 +28686,7 @@
         <v>72</v>
       </c>
       <c r="L163" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M163" t="s">
         <v>1237</v>
@@ -28745,7 +28751,7 @@
         <v>72</v>
       </c>
       <c r="L164" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M164" t="s">
         <v>1244</v>
@@ -28810,7 +28816,7 @@
         <v>72</v>
       </c>
       <c r="L165" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M165" t="s">
         <v>1251</v>
@@ -28875,7 +28881,7 @@
         <v>72</v>
       </c>
       <c r="L166" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M166" t="s">
         <v>1258</v>
@@ -28940,7 +28946,7 @@
         <v>72</v>
       </c>
       <c r="L167" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M167" t="s">
         <v>1265</v>
@@ -29005,7 +29011,7 @@
         <v>72</v>
       </c>
       <c r="L168" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M168" t="s">
         <v>1272</v>
@@ -29070,7 +29076,7 @@
         <v>72</v>
       </c>
       <c r="L169" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M169" t="s">
         <v>1279</v>
@@ -29135,7 +29141,7 @@
         <v>72</v>
       </c>
       <c r="L170" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M170" t="s">
         <v>1286</v>
@@ -29200,7 +29206,7 @@
         <v>72</v>
       </c>
       <c r="L171" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M171" t="s">
         <v>1293</v>
@@ -30386,7 +30392,7 @@
         <v>72</v>
       </c>
       <c r="L191" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M191" t="s">
         <v>578</v>
@@ -31790,7 +31796,7 @@
         <v>72</v>
       </c>
       <c r="L215" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M215" t="s">
         <v>578</v>
@@ -31852,7 +31858,7 @@
         <v>28</v>
       </c>
       <c r="L216" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q216" t="s">
         <v>567</v>
@@ -32510,7 +32516,7 @@
         <v>72</v>
       </c>
       <c r="L227" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M227" t="s">
         <v>578</v>
@@ -32572,7 +32578,7 @@
         <v>28</v>
       </c>
       <c r="L228" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q228" t="s">
         <v>567</v>
@@ -34609,7 +34615,7 @@
         <v>432</v>
       </c>
       <c r="L261" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M261" t="s">
         <v>125</v>
@@ -34674,7 +34680,7 @@
         <v>72</v>
       </c>
       <c r="L262" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M262" t="s">
         <v>578</v>
@@ -34789,7 +34795,7 @@
         <v>28</v>
       </c>
       <c r="L264" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q264" t="s">
         <v>567</v>
@@ -34910,7 +34916,7 @@
         <v>72</v>
       </c>
       <c r="L266" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M266" t="s">
         <v>125</v>
@@ -34978,7 +34984,7 @@
         <v>72</v>
       </c>
       <c r="L267" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M267" t="s">
         <v>125</v>
@@ -35046,7 +35052,7 @@
         <v>72</v>
       </c>
       <c r="L268" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M268" t="s">
         <v>125</v>
@@ -35114,7 +35120,7 @@
         <v>72</v>
       </c>
       <c r="L269" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M269" t="s">
         <v>125</v>
@@ -35250,7 +35256,7 @@
         <v>72</v>
       </c>
       <c r="L271" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M271" t="s">
         <v>125</v>
@@ -35318,7 +35324,7 @@
         <v>72</v>
       </c>
       <c r="L272" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M272" t="s">
         <v>125</v>
@@ -35386,7 +35392,7 @@
         <v>72</v>
       </c>
       <c r="L273" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M273" t="s">
         <v>125</v>
@@ -35454,7 +35460,7 @@
         <v>72</v>
       </c>
       <c r="L274" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M274" t="s">
         <v>125</v>
@@ -35522,7 +35528,7 @@
         <v>72</v>
       </c>
       <c r="L275" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M275" t="s">
         <v>125</v>
@@ -35590,7 +35596,7 @@
         <v>28</v>
       </c>
       <c r="L276" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="Q276" t="s">
         <v>1974</v>
@@ -35652,7 +35658,7 @@
         <v>28</v>
       </c>
       <c r="L277" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="Q277" t="s">
         <v>1974</v>
@@ -35714,7 +35720,7 @@
         <v>72</v>
       </c>
       <c r="L278" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M278" t="s">
         <v>125</v>
@@ -35782,7 +35788,7 @@
         <v>28</v>
       </c>
       <c r="L279" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="Q279" t="s">
         <v>1974</v>
@@ -36340,7 +36346,7 @@
         <v>432</v>
       </c>
       <c r="L288" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M288" t="s">
         <v>125</v>
@@ -36405,7 +36411,7 @@
         <v>72</v>
       </c>
       <c r="L289" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M289" t="s">
         <v>578</v>
@@ -36467,7 +36473,7 @@
         <v>72</v>
       </c>
       <c r="L290" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M290" t="s">
         <v>125</v>
@@ -36529,7 +36535,7 @@
         <v>72</v>
       </c>
       <c r="L291" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M291" t="s">
         <v>2078</v>
@@ -36594,7 +36600,7 @@
         <v>72</v>
       </c>
       <c r="L292" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M292" t="s">
         <v>125</v>
@@ -36656,7 +36662,7 @@
         <v>72</v>
       </c>
       <c r="L293" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M293" t="s">
         <v>125</v>
@@ -36718,7 +36724,7 @@
         <v>72</v>
       </c>
       <c r="L294" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M294" t="s">
         <v>125</v>
@@ -36780,7 +36786,7 @@
         <v>72</v>
       </c>
       <c r="L295" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M295" t="s">
         <v>125</v>
@@ -36842,7 +36848,7 @@
         <v>72</v>
       </c>
       <c r="L296" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M296" t="s">
         <v>125</v>
@@ -36904,7 +36910,7 @@
         <v>72</v>
       </c>
       <c r="L297" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M297" t="s">
         <v>125</v>
@@ -36966,7 +36972,7 @@
         <v>72</v>
       </c>
       <c r="L298" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M298" t="s">
         <v>125</v>
@@ -37028,7 +37034,7 @@
         <v>72</v>
       </c>
       <c r="L299" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M299" t="s">
         <v>125</v>
@@ -37090,7 +37096,7 @@
         <v>72</v>
       </c>
       <c r="L300" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M300" t="s">
         <v>125</v>
@@ -37152,7 +37158,7 @@
         <v>72</v>
       </c>
       <c r="L301" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M301" t="s">
         <v>125</v>
@@ -37214,7 +37220,7 @@
         <v>72</v>
       </c>
       <c r="L302" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M302" t="s">
         <v>125</v>
@@ -37276,7 +37282,7 @@
         <v>72</v>
       </c>
       <c r="L303" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M303" t="s">
         <v>125</v>
@@ -37338,7 +37344,7 @@
         <v>432</v>
       </c>
       <c r="L304" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M304" t="s">
         <v>2171</v>
@@ -37406,7 +37412,7 @@
         <v>432</v>
       </c>
       <c r="L305" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M305" t="s">
         <v>2181</v>
@@ -37474,7 +37480,7 @@
         <v>432</v>
       </c>
       <c r="L306" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M306" t="s">
         <v>2190</v>
@@ -37542,7 +37548,7 @@
         <v>432</v>
       </c>
       <c r="L307" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M307" t="s">
         <v>2199</v>
@@ -37610,7 +37616,7 @@
         <v>432</v>
       </c>
       <c r="L308" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M308" t="s">
         <v>2207</v>
@@ -37678,7 +37684,7 @@
         <v>72</v>
       </c>
       <c r="L309" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M309" t="s">
         <v>125</v>
@@ -37746,7 +37752,7 @@
         <v>432</v>
       </c>
       <c r="L310" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M310" t="s">
         <v>125</v>
@@ -37814,7 +37820,7 @@
         <v>72</v>
       </c>
       <c r="L311" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M311" t="s">
         <v>125</v>
@@ -39182,7 +39188,7 @@
         <v>432</v>
       </c>
       <c r="L332" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M332" t="s">
         <v>125</v>
@@ -39244,7 +39250,7 @@
         <v>72</v>
       </c>
       <c r="L333" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M333" t="s">
         <v>578</v>
@@ -39850,7 +39856,7 @@
         <v>72</v>
       </c>
       <c r="L342" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M342" t="s">
         <v>578</v>
@@ -40521,7 +40527,7 @@
         <v>72</v>
       </c>
       <c r="L352" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M352" t="s">
         <v>578</v>
@@ -40583,7 +40589,7 @@
         <v>72</v>
       </c>
       <c r="L353" t="s">
-        <v>49</v>
+        <v>5728</v>
       </c>
       <c r="M353" t="s">
         <v>2564</v>
@@ -40648,7 +40654,7 @@
         <v>72</v>
       </c>
       <c r="L354" t="s">
-        <v>49</v>
+        <v>5728</v>
       </c>
       <c r="M354" t="s">
         <v>2573</v>
@@ -40775,7 +40781,7 @@
         <v>432</v>
       </c>
       <c r="L356" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M356" t="s">
         <v>2588</v>
@@ -40849,7 +40855,7 @@
         <v>432</v>
       </c>
       <c r="L357" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M357" t="s">
         <v>2599</v>
@@ -40923,7 +40929,7 @@
         <v>432</v>
       </c>
       <c r="L358" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M358" t="s">
         <v>2599</v>
@@ -41047,7 +41053,7 @@
         <v>72</v>
       </c>
       <c r="L360" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M360" t="s">
         <v>578</v>
@@ -41109,7 +41115,7 @@
         <v>72</v>
       </c>
       <c r="L361" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M361" t="s">
         <v>2630</v>
@@ -41174,7 +41180,7 @@
         <v>72</v>
       </c>
       <c r="L362" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M362" t="s">
         <v>2640</v>
@@ -41242,7 +41248,7 @@
         <v>72</v>
       </c>
       <c r="L363" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M363" t="s">
         <v>2650</v>
@@ -41310,7 +41316,7 @@
         <v>72</v>
       </c>
       <c r="L364" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M364" t="s">
         <v>125</v>
@@ -41372,7 +41378,7 @@
         <v>72</v>
       </c>
       <c r="L365" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M365" t="s">
         <v>125</v>
@@ -41434,7 +41440,7 @@
         <v>72</v>
       </c>
       <c r="L366" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M366" t="s">
         <v>125</v>
@@ -41496,7 +41502,7 @@
         <v>72</v>
       </c>
       <c r="L367" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M367" t="s">
         <v>125</v>
@@ -41558,7 +41564,7 @@
         <v>72</v>
       </c>
       <c r="L368" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M368" t="s">
         <v>125</v>
@@ -41620,7 +41626,7 @@
         <v>72</v>
       </c>
       <c r="L369" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M369" t="s">
         <v>125</v>
@@ -41682,7 +41688,7 @@
         <v>72</v>
       </c>
       <c r="L370" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M370" t="s">
         <v>125</v>
@@ -41744,7 +41750,7 @@
         <v>72</v>
       </c>
       <c r="L371" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M371" t="s">
         <v>125</v>
@@ -41806,7 +41812,7 @@
         <v>72</v>
       </c>
       <c r="L372" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M372" t="s">
         <v>125</v>
@@ -41868,7 +41874,7 @@
         <v>72</v>
       </c>
       <c r="L373" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M373" t="s">
         <v>125</v>
@@ -42550,7 +42556,7 @@
         <v>72</v>
       </c>
       <c r="L384" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M384" t="s">
         <v>578</v>
@@ -42612,7 +42618,7 @@
         <v>72</v>
       </c>
       <c r="L385" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M385" t="s">
         <v>2812</v>
@@ -42969,7 +42975,7 @@
         <v>72</v>
       </c>
       <c r="L391" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M391" t="s">
         <v>578</v>
@@ -43031,7 +43037,7 @@
         <v>28</v>
       </c>
       <c r="L392" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="P392" t="s">
         <v>2862</v>
@@ -43090,7 +43096,7 @@
         <v>28</v>
       </c>
       <c r="L393" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="P393" t="s">
         <v>2862</v>
@@ -43149,7 +43155,7 @@
         <v>28</v>
       </c>
       <c r="L394" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="P394" t="s">
         <v>2862</v>
@@ -43208,7 +43214,7 @@
         <v>28</v>
       </c>
       <c r="L395" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="P395" t="s">
         <v>2862</v>
@@ -43267,7 +43273,7 @@
         <v>28</v>
       </c>
       <c r="L396" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="P396" t="s">
         <v>2862</v>
@@ -43326,7 +43332,7 @@
         <v>28</v>
       </c>
       <c r="L397" t="s">
-        <v>1714</v>
+        <v>5731</v>
       </c>
       <c r="P397" t="s">
         <v>2862</v>
@@ -44113,7 +44119,7 @@
         <v>72</v>
       </c>
       <c r="L411" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M411" t="s">
         <v>578</v>
@@ -44175,7 +44181,7 @@
         <v>72</v>
       </c>
       <c r="L412" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M412" t="s">
         <v>125</v>
@@ -44237,7 +44243,7 @@
         <v>72</v>
       </c>
       <c r="L413" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M413" t="s">
         <v>125</v>
@@ -44299,7 +44305,7 @@
         <v>72</v>
       </c>
       <c r="L414" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M414" t="s">
         <v>125</v>
@@ -44361,7 +44367,7 @@
         <v>72</v>
       </c>
       <c r="L415" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M415" t="s">
         <v>125</v>
@@ -44423,7 +44429,7 @@
         <v>72</v>
       </c>
       <c r="L416" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M416" t="s">
         <v>125</v>
@@ -44485,7 +44491,7 @@
         <v>72</v>
       </c>
       <c r="L417" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M417" t="s">
         <v>125</v>
@@ -44547,7 +44553,7 @@
         <v>72</v>
       </c>
       <c r="L418" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M418" t="s">
         <v>125</v>
@@ -44609,7 +44615,7 @@
         <v>72</v>
       </c>
       <c r="L419" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M419" t="s">
         <v>125</v>
@@ -44671,7 +44677,7 @@
         <v>72</v>
       </c>
       <c r="L420" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M420" t="s">
         <v>125</v>
@@ -44733,7 +44739,7 @@
         <v>72</v>
       </c>
       <c r="L421" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M421" t="s">
         <v>125</v>
@@ -44795,7 +44801,7 @@
         <v>72</v>
       </c>
       <c r="L422" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M422" t="s">
         <v>125</v>
@@ -44857,7 +44863,7 @@
         <v>72</v>
       </c>
       <c r="L423" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M423" t="s">
         <v>125</v>
@@ -47922,7 +47928,7 @@
         <v>72</v>
       </c>
       <c r="L475" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M475" t="s">
         <v>578</v>
@@ -47984,7 +47990,7 @@
         <v>72</v>
       </c>
       <c r="L476" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M476" t="s">
         <v>125</v>
@@ -48108,7 +48114,7 @@
         <v>72</v>
       </c>
       <c r="L478" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M478" t="s">
         <v>125</v>
@@ -48234,6 +48240,9 @@
       <c r="K480" t="s">
         <v>28</v>
       </c>
+      <c r="L480" t="s">
+        <v>1714</v>
+      </c>
       <c r="P480" t="s">
         <v>3437</v>
       </c>
@@ -48355,6 +48364,9 @@
       <c r="K482" t="s">
         <v>28</v>
       </c>
+      <c r="L482" t="s">
+        <v>1714</v>
+      </c>
       <c r="P482" t="s">
         <v>3452</v>
       </c>
@@ -48533,7 +48545,7 @@
         <v>72</v>
       </c>
       <c r="L485" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M485" t="s">
         <v>578</v>
@@ -48648,7 +48660,7 @@
         <v>72</v>
       </c>
       <c r="L487" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M487" t="s">
         <v>3489</v>
@@ -48713,7 +48725,7 @@
         <v>72</v>
       </c>
       <c r="L488" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M488" t="s">
         <v>578</v>
@@ -48775,7 +48787,7 @@
         <v>72</v>
       </c>
       <c r="L489" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M489" t="s">
         <v>125</v>
@@ -48843,7 +48855,7 @@
         <v>72</v>
       </c>
       <c r="L490" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M490" t="s">
         <v>125</v>
@@ -49212,7 +49224,7 @@
         <v>72</v>
       </c>
       <c r="L496" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M496" t="s">
         <v>578</v>
@@ -49274,7 +49286,7 @@
         <v>72</v>
       </c>
       <c r="L497" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M497" t="s">
         <v>125</v>
@@ -49345,7 +49357,7 @@
         <v>72</v>
       </c>
       <c r="L498" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M498" t="s">
         <v>125</v>
@@ -49599,7 +49611,7 @@
         <v>432</v>
       </c>
       <c r="L502" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M502" t="s">
         <v>3540</v>
@@ -49947,7 +49959,7 @@
         <v>72</v>
       </c>
       <c r="L508" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M508" t="s">
         <v>578</v>
@@ -50009,7 +50021,7 @@
         <v>72</v>
       </c>
       <c r="L509" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M509" t="s">
         <v>125</v>
@@ -50080,7 +50092,7 @@
         <v>72</v>
       </c>
       <c r="L510" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M510" t="s">
         <v>125</v>
@@ -50325,7 +50337,7 @@
         <v>432</v>
       </c>
       <c r="L514" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M514" t="s">
         <v>3540</v>
@@ -50508,7 +50520,7 @@
         <v>432</v>
       </c>
       <c r="L517" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M517" t="s">
         <v>3540</v>
@@ -50694,7 +50706,7 @@
         <v>72</v>
       </c>
       <c r="L520" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M520" t="s">
         <v>578</v>
@@ -50756,7 +50768,7 @@
         <v>72</v>
       </c>
       <c r="L521" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M521" t="s">
         <v>125</v>
@@ -50827,7 +50839,7 @@
         <v>72</v>
       </c>
       <c r="L522" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M522" t="s">
         <v>125</v>
@@ -51137,7 +51149,7 @@
         <v>432</v>
       </c>
       <c r="L527" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M527" t="s">
         <v>3540</v>
@@ -51261,7 +51273,7 @@
         <v>72</v>
       </c>
       <c r="L529" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M529" t="s">
         <v>578</v>
@@ -51323,7 +51335,7 @@
         <v>72</v>
       </c>
       <c r="L530" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M530" t="s">
         <v>125</v>
@@ -51391,7 +51403,7 @@
         <v>72</v>
       </c>
       <c r="L531" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M531" t="s">
         <v>125</v>
@@ -51804,7 +51816,7 @@
         <v>432</v>
       </c>
       <c r="L538" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M538" t="s">
         <v>3836</v>
@@ -52046,7 +52058,7 @@
         <v>72</v>
       </c>
       <c r="L542" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M542" t="s">
         <v>3863</v>
@@ -52170,7 +52182,7 @@
         <v>432</v>
       </c>
       <c r="L544" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M544" t="s">
         <v>3836</v>
@@ -52297,7 +52309,7 @@
         <v>432</v>
       </c>
       <c r="L546" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M546" t="s">
         <v>3891</v>
@@ -52424,7 +52436,7 @@
         <v>72</v>
       </c>
       <c r="L548" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M548" t="s">
         <v>578</v>
@@ -52486,7 +52498,7 @@
         <v>72</v>
       </c>
       <c r="L549" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M549" t="s">
         <v>125</v>
@@ -52551,7 +52563,7 @@
         <v>72</v>
       </c>
       <c r="L550" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M550" t="s">
         <v>125</v>
@@ -52616,7 +52628,7 @@
         <v>432</v>
       </c>
       <c r="L551" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M551" t="s">
         <v>3931</v>
@@ -53369,7 +53381,7 @@
         <v>72</v>
       </c>
       <c r="L563" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M563" t="s">
         <v>578</v>
@@ -53431,7 +53443,7 @@
         <v>72</v>
       </c>
       <c r="L564" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M564" t="s">
         <v>125</v>
@@ -53782,7 +53794,7 @@
         <v>72</v>
       </c>
       <c r="L570" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M570" t="s">
         <v>423</v>
@@ -55765,7 +55777,7 @@
         <v>432</v>
       </c>
       <c r="L600" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M600" t="s">
         <v>4233</v>
@@ -56297,7 +56309,7 @@
         <v>72</v>
       </c>
       <c r="L608" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M608" t="s">
         <v>125</v>
@@ -56418,7 +56430,7 @@
         <v>72</v>
       </c>
       <c r="L610" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M610" t="s">
         <v>125</v>
@@ -56536,7 +56548,7 @@
         <v>72</v>
       </c>
       <c r="L612" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M612" t="s">
         <v>578</v>
@@ -56598,7 +56610,7 @@
         <v>28</v>
       </c>
       <c r="L613" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q613" t="s">
         <v>567</v>
@@ -56660,7 +56672,7 @@
         <v>72</v>
       </c>
       <c r="L614" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M614" t="s">
         <v>4321</v>
@@ -56840,7 +56852,7 @@
         <v>72</v>
       </c>
       <c r="L617" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M617" t="s">
         <v>125</v>
@@ -57398,7 +57410,7 @@
         <v>72</v>
       </c>
       <c r="L626" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M626" t="s">
         <v>125</v>
@@ -57460,7 +57472,7 @@
         <v>72</v>
       </c>
       <c r="L627" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M627" t="s">
         <v>125</v>
@@ -57522,7 +57534,7 @@
         <v>72</v>
       </c>
       <c r="L628" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M628" t="s">
         <v>125</v>
@@ -57584,7 +57596,7 @@
         <v>72</v>
       </c>
       <c r="L629" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M629" t="s">
         <v>125</v>
@@ -57646,7 +57658,7 @@
         <v>72</v>
       </c>
       <c r="L630" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M630" t="s">
         <v>125</v>
@@ -57708,7 +57720,7 @@
         <v>72</v>
       </c>
       <c r="L631" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M631" t="s">
         <v>125</v>
@@ -57770,7 +57782,7 @@
         <v>72</v>
       </c>
       <c r="L632" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M632" t="s">
         <v>125</v>
@@ -57832,7 +57844,7 @@
         <v>72</v>
       </c>
       <c r="L633" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M633" t="s">
         <v>125</v>
@@ -57894,7 +57906,7 @@
         <v>72</v>
       </c>
       <c r="L634" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M634" t="s">
         <v>125</v>
@@ -57956,7 +57968,7 @@
         <v>72</v>
       </c>
       <c r="L635" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M635" t="s">
         <v>125</v>
@@ -58018,7 +58030,7 @@
         <v>72</v>
       </c>
       <c r="L636" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M636" t="s">
         <v>125</v>
@@ -58080,7 +58092,7 @@
         <v>72</v>
       </c>
       <c r="L637" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M637" t="s">
         <v>125</v>
@@ -58142,7 +58154,7 @@
         <v>72</v>
       </c>
       <c r="L638" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M638" t="s">
         <v>125</v>
@@ -58260,7 +58272,7 @@
         <v>72</v>
       </c>
       <c r="L640" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M640" t="s">
         <v>125</v>
@@ -58325,7 +58337,7 @@
         <v>432</v>
       </c>
       <c r="L641" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M641" t="s">
         <v>4501</v>
@@ -58393,7 +58405,7 @@
         <v>72</v>
       </c>
       <c r="L642" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M642" t="s">
         <v>557</v>
@@ -58455,7 +58467,7 @@
         <v>72</v>
       </c>
       <c r="L643" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M643" t="s">
         <v>125</v>
@@ -58517,7 +58529,7 @@
         <v>72</v>
       </c>
       <c r="L644" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M644" t="s">
         <v>578</v>
@@ -58966,7 +58978,7 @@
         <v>432</v>
       </c>
       <c r="L651" t="s">
-        <v>5731</v>
+        <v>5730</v>
       </c>
       <c r="M651" t="s">
         <v>4578</v>
@@ -59229,7 +59241,7 @@
         <v>432</v>
       </c>
       <c r="L655" t="s">
-        <v>5731</v>
+        <v>5730</v>
       </c>
       <c r="M655" t="s">
         <v>4609</v>
@@ -60024,7 +60036,7 @@
         <v>72</v>
       </c>
       <c r="L667" t="s">
-        <v>5731</v>
+        <v>5730</v>
       </c>
       <c r="M667" t="s">
         <v>4700</v>
@@ -60213,7 +60225,7 @@
         <v>72</v>
       </c>
       <c r="L670" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M670" t="s">
         <v>125</v>
@@ -60278,7 +60290,7 @@
         <v>432</v>
       </c>
       <c r="L671" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M671" t="s">
         <v>125</v>
@@ -60467,7 +60479,7 @@
         <v>432</v>
       </c>
       <c r="L674" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M674" t="s">
         <v>4750</v>
@@ -60535,7 +60547,7 @@
         <v>432</v>
       </c>
       <c r="L675" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M675" t="s">
         <v>4759</v>
@@ -60727,7 +60739,7 @@
         <v>432</v>
       </c>
       <c r="L678" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M678" t="s">
         <v>4779</v>
@@ -60795,7 +60807,7 @@
         <v>432</v>
       </c>
       <c r="L679" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M679" t="s">
         <v>4788</v>
@@ -60863,7 +60875,7 @@
         <v>432</v>
       </c>
       <c r="L680" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M680" t="s">
         <v>4797</v>
@@ -60928,7 +60940,7 @@
         <v>432</v>
       </c>
       <c r="L681" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M681" t="s">
         <v>125</v>
@@ -61049,7 +61061,7 @@
         <v>72</v>
       </c>
       <c r="L683" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M683" t="s">
         <v>578</v>
@@ -61229,7 +61241,7 @@
         <v>72</v>
       </c>
       <c r="L686" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M686" t="s">
         <v>125</v>
@@ -61297,7 +61309,7 @@
         <v>72</v>
       </c>
       <c r="L687" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M687" t="s">
         <v>125</v>
@@ -61536,7 +61548,7 @@
         <v>72</v>
       </c>
       <c r="L691" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M691" t="s">
         <v>125</v>
@@ -61604,7 +61616,7 @@
         <v>72</v>
       </c>
       <c r="L692" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M692" t="s">
         <v>125</v>
@@ -62053,7 +62065,7 @@
         <v>72</v>
       </c>
       <c r="L699" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M699" t="s">
         <v>125</v>
@@ -62513,7 +62525,7 @@
         <v>72</v>
       </c>
       <c r="L707" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M707" t="s">
         <v>125</v>
@@ -62575,7 +62587,7 @@
         <v>72</v>
       </c>
       <c r="L708" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M708" t="s">
         <v>125</v>
@@ -62696,7 +62708,7 @@
         <v>72</v>
       </c>
       <c r="L710" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M710" t="s">
         <v>125</v>
@@ -62761,7 +62773,7 @@
         <v>72</v>
       </c>
       <c r="L711" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M711" t="s">
         <v>125</v>
@@ -62885,7 +62897,7 @@
         <v>72</v>
       </c>
       <c r="L713" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M713" t="s">
         <v>125</v>
@@ -63015,7 +63027,7 @@
         <v>72</v>
       </c>
       <c r="L715" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M715" t="s">
         <v>125</v>
@@ -63204,7 +63216,7 @@
         <v>72</v>
       </c>
       <c r="L718" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M718" t="s">
         <v>125</v>
@@ -63272,7 +63284,7 @@
         <v>72</v>
       </c>
       <c r="L719" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M719" t="s">
         <v>125</v>
@@ -63526,7 +63538,7 @@
         <v>72</v>
       </c>
       <c r="L723" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M723" t="s">
         <v>125</v>
@@ -63594,7 +63606,7 @@
         <v>72</v>
       </c>
       <c r="L724" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M724" t="s">
         <v>125</v>
@@ -63718,7 +63730,7 @@
         <v>72</v>
       </c>
       <c r="L726" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M726" t="s">
         <v>578</v>
@@ -63780,7 +63792,7 @@
         <v>28</v>
       </c>
       <c r="L727" t="s">
-        <v>180</v>
+        <v>1714</v>
       </c>
       <c r="Q727" t="s">
         <v>567</v>
@@ -64013,7 +64025,7 @@
         <v>72</v>
       </c>
       <c r="L731" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M731" t="s">
         <v>125</v>
@@ -64137,7 +64149,7 @@
         <v>72</v>
       </c>
       <c r="L733" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M733" t="s">
         <v>125</v>
@@ -64264,7 +64276,7 @@
         <v>72</v>
       </c>
       <c r="L735" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M735" t="s">
         <v>125</v>
@@ -64391,7 +64403,7 @@
         <v>72</v>
       </c>
       <c r="L737" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M737" t="s">
         <v>125</v>
@@ -64518,7 +64530,7 @@
         <v>72</v>
       </c>
       <c r="L739" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M739" t="s">
         <v>125</v>
@@ -64645,7 +64657,7 @@
         <v>72</v>
       </c>
       <c r="L741" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M741" t="s">
         <v>125</v>
@@ -64772,7 +64784,7 @@
         <v>72</v>
       </c>
       <c r="L743" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M743" t="s">
         <v>125</v>
@@ -64899,7 +64911,7 @@
         <v>72</v>
       </c>
       <c r="L745" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M745" t="s">
         <v>125</v>
@@ -65026,7 +65038,7 @@
         <v>72</v>
       </c>
       <c r="L747" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M747" t="s">
         <v>125</v>
@@ -65153,7 +65165,7 @@
         <v>72</v>
       </c>
       <c r="L749" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M749" t="s">
         <v>125</v>
@@ -65221,7 +65233,7 @@
         <v>72</v>
       </c>
       <c r="L750" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M750" t="s">
         <v>125</v>
@@ -65584,7 +65596,7 @@
         <v>72</v>
       </c>
       <c r="L756" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M756" t="s">
         <v>5332</v>
@@ -65770,7 +65782,7 @@
         <v>72</v>
       </c>
       <c r="L759" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M759" t="s">
         <v>125</v>
@@ -65838,7 +65850,7 @@
         <v>432</v>
       </c>
       <c r="L760" t="s">
-        <v>5728</v>
+        <v>5730</v>
       </c>
       <c r="M760" t="s">
         <v>5358</v>
@@ -65965,7 +65977,7 @@
         <v>72</v>
       </c>
       <c r="L762" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M762" t="s">
         <v>125</v>
@@ -66092,7 +66104,7 @@
         <v>72</v>
       </c>
       <c r="L764" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M764" t="s">
         <v>125</v>
@@ -66219,7 +66231,7 @@
         <v>72</v>
       </c>
       <c r="L766" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M766" t="s">
         <v>578</v>
@@ -66281,7 +66293,7 @@
         <v>72</v>
       </c>
       <c r="L767" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M767" t="s">
         <v>5411</v>
@@ -66476,7 +66488,7 @@
         <v>72</v>
       </c>
       <c r="L770" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M770" t="s">
         <v>125</v>
@@ -66600,7 +66612,7 @@
         <v>72</v>
       </c>
       <c r="L772" t="s">
-        <v>5728</v>
+        <v>36</v>
       </c>
       <c r="M772" t="s">
         <v>5450</v>
@@ -66727,7 +66739,7 @@
         <v>72</v>
       </c>
       <c r="L774" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M774" t="s">
         <v>578</v>
@@ -66848,7 +66860,7 @@
         <v>432</v>
       </c>
       <c r="L776" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M776" t="s">
         <v>5481</v>
@@ -67146,7 +67158,7 @@
         <v>72</v>
       </c>
       <c r="L781" t="s">
-        <v>5728</v>
+        <v>49</v>
       </c>
       <c r="M781" t="s">
         <v>578</v>

</xml_diff>